<commit_message>
Actualización: Puesta en marcha
</commit_message>
<xml_diff>
--- a/data/data_final.xlsx
+++ b/data/data_final.xlsx
@@ -929,7 +929,7 @@
         <v>3500</v>
       </c>
       <c r="AD2" t="n">
-        <v>360.3</v>
+        <v>514.2</v>
       </c>
       <c r="AE2" t="n">
         <v>4</v>
@@ -953,7 +953,7 @@
         <v>3472</v>
       </c>
       <c r="AL2" t="n">
-        <v>349.7</v>
+        <v>548.3</v>
       </c>
       <c r="AM2" t="n">
         <v>5</v>
@@ -977,7 +977,7 @@
         <v>3592</v>
       </c>
       <c r="AT2" t="n">
-        <v>379.2</v>
+        <v>536.2</v>
       </c>
       <c r="AU2" t="n">
         <v>5</v>
@@ -1037,7 +1037,7 @@
         <v>73.45840544468858</v>
       </c>
       <c r="BN2" t="n">
-        <v>20.44</v>
+        <v>30</v>
       </c>
       <c r="BO2" t="n">
         <v>73.00333498511715</v>
@@ -1198,7 +1198,7 @@
         <v>3654</v>
       </c>
       <c r="AD3" t="n">
-        <v>297.1</v>
+        <v>228.8</v>
       </c>
       <c r="AE3" t="n">
         <v>4</v>
@@ -1222,7 +1222,7 @@
         <v>3655</v>
       </c>
       <c r="AL3" t="n">
-        <v>294.9</v>
+        <v>252</v>
       </c>
       <c r="AM3" t="n">
         <v>4</v>
@@ -1246,7 +1246,7 @@
         <v>3676</v>
       </c>
       <c r="AT3" t="n">
-        <v>310.7</v>
+        <v>230.1</v>
       </c>
       <c r="AU3" t="n">
         <v>4</v>
@@ -1306,7 +1306,7 @@
         <v>136.4879413130573</v>
       </c>
       <c r="BN3" t="n">
-        <v>36.82</v>
+        <v>29</v>
       </c>
       <c r="BO3" t="n">
         <v>133.4956822331906</v>
@@ -1467,7 +1467,7 @@
         <v>3548</v>
       </c>
       <c r="AD4" t="n">
-        <v>363.8</v>
+        <v>250.4</v>
       </c>
       <c r="AE4" t="n">
         <v>2</v>
@@ -1491,7 +1491,7 @@
         <v>3659</v>
       </c>
       <c r="AL4" t="n">
-        <v>342.6</v>
+        <v>244.2</v>
       </c>
       <c r="AM4" t="n">
         <v>2</v>
@@ -1515,7 +1515,7 @@
         <v>3578</v>
       </c>
       <c r="AT4" t="n">
-        <v>366.3</v>
+        <v>241.7</v>
       </c>
       <c r="AU4" t="n">
         <v>2</v>
@@ -1579,7 +1579,7 @@
         </is>
       </c>
       <c r="BN4" t="n">
-        <v>43.71</v>
+        <v>30</v>
       </c>
       <c r="BO4" t="n">
         <v>158.4734942461915</v>
@@ -1742,7 +1742,7 @@
         <v>3567</v>
       </c>
       <c r="AD5" t="n">
-        <v>384.5</v>
+        <v>372.4</v>
       </c>
       <c r="AE5" t="n">
         <v>2</v>
@@ -1766,7 +1766,7 @@
         <v>3567</v>
       </c>
       <c r="AL5" t="n">
-        <v>372.4</v>
+        <v>361.6</v>
       </c>
       <c r="AM5" t="n">
         <v>2</v>
@@ -1790,7 +1790,7 @@
         <v>3675</v>
       </c>
       <c r="AT5" t="n">
-        <v>369.4</v>
+        <v>392.2</v>
       </c>
       <c r="AU5" t="n">
         <v>2</v>
@@ -2011,7 +2011,7 @@
         <v>3465</v>
       </c>
       <c r="AD6" t="n">
-        <v>351.8</v>
+        <v>336</v>
       </c>
       <c r="AE6" t="n">
         <v>2</v>
@@ -2035,7 +2035,7 @@
         <v>3564</v>
       </c>
       <c r="AL6" t="n">
-        <v>325.7</v>
+        <v>338.4</v>
       </c>
       <c r="AM6" t="n">
         <v>2</v>
@@ -2059,7 +2059,7 @@
         <v>3653</v>
       </c>
       <c r="AT6" t="n">
-        <v>327.5</v>
+        <v>330.5</v>
       </c>
       <c r="AU6" t="n">
         <v>2</v>
@@ -2280,7 +2280,7 @@
         <v>3500</v>
       </c>
       <c r="AD7" t="n">
-        <v>192.6</v>
+        <v>179.3</v>
       </c>
       <c r="AE7" t="n">
         <v>5</v>
@@ -2304,7 +2304,7 @@
         <v>3478</v>
       </c>
       <c r="AL7" t="n">
-        <v>183.9</v>
+        <v>196</v>
       </c>
       <c r="AM7" t="n">
         <v>4</v>
@@ -2328,7 +2328,7 @@
         <v>3500</v>
       </c>
       <c r="AT7" t="n">
-        <v>169.1</v>
+        <v>170.2</v>
       </c>
       <c r="AU7" t="n">
         <v>5</v>
@@ -2547,7 +2547,7 @@
         <v>3655</v>
       </c>
       <c r="AD8" t="n">
-        <v>231.7</v>
+        <v>217.4</v>
       </c>
       <c r="AE8" t="n">
         <v>2</v>
@@ -2571,7 +2571,7 @@
         <v>3655</v>
       </c>
       <c r="AL8" t="n">
-        <v>207.5</v>
+        <v>224</v>
       </c>
       <c r="AM8" t="n">
         <v>2</v>
@@ -2595,7 +2595,7 @@
         <v>3548</v>
       </c>
       <c r="AT8" t="n">
-        <v>207.9</v>
+        <v>205.6</v>
       </c>
       <c r="AU8" t="n">
         <v>2</v>

</xml_diff>